<commit_message>
chore(assets): standardize runtime asset names
Document asset naming rules, add card-art validation, and move non-runtime Docs import files into archive storage.
</commit_message>
<xml_diff>
--- a/project-a/tables/excel/CharacterCards.xlsx
+++ b/project-a/tables/excel/CharacterCards.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="character_cards" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="card_effects" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="character_cards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effects" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: drive Tsuki card motions from table
</commit_message>
<xml_diff>
--- a/project-a/tables/excel/CharacterCards.xlsx
+++ b/project-a/tables/excel/CharacterCards.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -422,11 +422,12 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -463,25 +464,30 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>motion_animation</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>text</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>copies</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>keywords[]</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>effects</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>inspiration</t>
         </is>
@@ -520,20 +526,25 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>int</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>json,null</t>
         </is>
@@ -590,6 +601,11 @@
           <t>data</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -617,14 +633,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>피해 100%.</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>2</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>[{"type": "damage", "percent": 100, "target": "enemy"}]</t>
         </is>
@@ -656,14 +677,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>피해 220%.</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
         <is>
           <t>[{"type": "damage", "percent": 220, "target": "enemy"}]</t>
         </is>
@@ -695,14 +721,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>실드 100%.</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
         <is>
           <t>[{"type": "shield", "percent": 100, "target": "self"}]</t>
         </is>
@@ -734,14 +765,19 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>자신의 공격 카드 드로우 1. 1턴간 자신의 공격 카드 피해량 40% 증가.</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
         <is>
           <t>[{"type": "draw", "card_type": "attack", "amount": 1}, {"type": "buff", "buff": "attack_damage_up", "percent": 40, "duration_turns": 1, "scope": "own_attack"}]</t>
         </is>
@@ -773,23 +809,28 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>모든 적 피해 220%. 영감: 비용 1 감소.</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>영감</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>[{"type": "damage", "percent": 220, "target": "all_enemies"}]</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>[{"type": "cost_delta", "amount": -1}]</t>
         </is>
@@ -821,18 +862,23 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>[보존] 피해 180%. 핸드의 무작위 자신의 카드 1장의 영감 효과를 활성화.</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>보존</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>[{"type": "damage", "percent": 180, "target": "enemy"}, {"type": "activate_inspiration", "target": "random_own_in_hand", "amount": 1}]</t>
         </is>
@@ -864,18 +910,23 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>[유일] 자신의 영감 효과가 활성화된 카드 사용 시 모든 적에게 피해 120%.</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>유일</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>[{"type": "passive", "trigger": "on_play_inspired_card", "effect": {"type": "damage", "percent": 120, "target": "all_enemies"}}]</t>
         </is>
@@ -907,23 +958,28 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>모든 적 피해 180%. 영감: 타격 1회 추가, 피해량 20% 감소.</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>1</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>영감</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>[{"type": "damage", "percent": 180, "target": "all_enemies"}]</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>[{"type": "add_hit", "amount": 1}, {"type": "damage_delta", "percent": -20}]</t>
         </is>

</xml_diff>

<commit_message>
refactor(tables): normalize card effect rows
</commit_message>
<xml_diff>
--- a/project-a/tables/excel/CharacterCards.xlsx
+++ b/project-a/tables/excel/CharacterCards.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="character_cards" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effects" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effect_rows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="card_effects" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,20 +415,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="52" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -439,71 +439,66 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>card_key</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>character</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>cost</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>card_type</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>motion_animation</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>text_template</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>copies</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>keywords[]</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>effects</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>inspiration</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
+          <t>key,string</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>string</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>key,string</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>string</t>
@@ -511,42 +506,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>int</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>string</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>json,null</t>
         </is>
       </c>
     </row>
@@ -601,387 +591,372 @@
           <t>data</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
+          <t>tsuki/long_sword_slash</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>long_sword_slash</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>장검 베기</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>attack</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>피해 100%.</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>피해 {0}%.</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
         <v>2</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>[{"type": "damage", "percent": 100, "target": "enemy"}]</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
+          <t>tsuki/high_speed_slash</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>high_speed_slash</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>고속 베기</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>attack</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>피해 220%.</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>피해 {0}%.</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>[{"type": "damage", "percent": 220, "target": "enemy"}]</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
+          <t>tsuki/let_flow</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>let_flow</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>흘려 보내기</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>skill</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Idle</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>실드 100%.</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>실드 {0}%.</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>[{"type": "shield", "percent": 100, "target": "self"}]</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
+          <t>tsuki/suppress_ready</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>suppress_ready</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>제압 준비</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>skill</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Idle</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>자신의 공격 카드 드로우 1. 1턴간 자신의 공격 카드 피해량 40% 증가.</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>자신의 공격 카드 드로우 {0}. {2}턴간 자신의 공격 카드 피해량 {1}% 증가.</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>[{"type": "draw", "card_type": "attack", "amount": 1}, {"type": "buff", "buff": "attack_damage_up", "percent": 40, "duration_turns": 1, "scope": "own_attack"}]</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
+          <t>tsuki/steal_slash</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>steal_slash</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>훔쳐베기</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>2</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>attack</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>모든 적 피해 220%. 영감: 비용 1 감소.</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>모든 적 피해 {0}%. 영감: 비용 {1} 감소.</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>영감</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>[{"type": "damage", "percent": 220, "target": "all_enemies"}]</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>[{"type": "cost_delta", "amount": -1}]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
+          <t>tsuki/feint_strike</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>feint_strike</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>눈속임 일격</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>attack</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>[보존] 피해 180%. 핸드의 무작위 자신의 카드 1장의 영감 효과를 활성화.</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>[보존] 피해 {0}%. 핸드의 무작위 자신의 카드 {1}장의 영감 효과를 활성화.</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>보존</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>[{"type": "damage", "percent": 180, "target": "enemy"}, {"type": "activate_inspiration", "target": "random_own_in_hand", "amount": 1}]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
+          <t>tsuki/freezing_blade</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>freezing_blade</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>빙점 칼날</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>enhance</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Idle</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>[유일] 자신의 영감 효과가 활성화된 카드 사용 시 모든 적에게 피해 120%.</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>[유일] 자신의 영감 효과가 활성화된 카드 사용 시 모든 적에게 피해 {0}%.</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>유일</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>[{"type": "passive", "trigger": "on_play_inspired_card", "effect": {"type": "damage", "percent": 120, "target": "all_enemies"}}]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
+          <t>tsuki/iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>tsuki</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>iceberg_cleave</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>빙산 가르기</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>attack</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>모든 적 피해 180%. 영감: 타격 1회 추가, 피해량 20% 감소.</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>모든 적 피해 {0}%. 영감: 타격 {1}회 추가, 피해량 {2}% 감소.</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>영감</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>[{"type": "damage", "percent": 180, "target": "all_enemies"}]</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>[{"type": "add_hit", "amount": 1}, {"type": "damage_delta", "percent": -20}]</t>
         </is>
       </c>
     </row>
@@ -991,6 +966,895 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>#data</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>card_key</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>character</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>card_id</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>effect_type</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>card_type</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>buff</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>duration_turns</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>child_effect_type</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>child_target</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>child_percent</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>text_arg_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>key,string</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>int,null</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>int,null</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>int,null</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>int,null</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>int,null</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tsuki_long_sword_slash_damage</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tsuki/long_sword_slash</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>long_sword_slash</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>100</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tsuki_high_speed_slash_damage</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>tsuki/high_speed_slash</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>high_speed_slash</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>220</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tsuki_let_flow_shield</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>tsuki/let_flow</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>let_flow</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>100</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tsuki_suppress_ready_draw</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>tsuki/suppress_ready</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>suppress_ready</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tsuki_suppress_ready_attack_buff</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>tsuki/suppress_ready</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>suppress_ready</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>buff</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>attack_damage_up</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>40</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>own_attack</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>tsuki_suppress_ready_buff_turns_text</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>tsuki/suppress_ready</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>suppress_ready</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>text_only</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tsuki_steal_slash_damage</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>tsuki/steal_slash</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>steal_slash</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>all_enemies</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>220</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tsuki_steal_slash_inspiration_cost</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>tsuki/steal_slash</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>steal_slash</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>on_inspiration</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>cost_delta</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tsuki_feint_strike_damage</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>tsuki/feint_strike</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>feint_strike</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>180</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tsuki_feint_strike_activate_inspiration</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>tsuki/feint_strike</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>feint_strike</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>activate_inspiration</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>random_own_in_hand</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tsuki_freezing_blade_passive_damage</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>tsuki/freezing_blade</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>freezing_blade</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>on_play_inspired_card</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>all_enemies</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>120</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tsuki_iceberg_cleave_damage</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>tsuki/iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>all_enemies</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>180</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tsuki_iceberg_cleave_extra_hit</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>tsuki/iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>on_inspiration</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>add_hit</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tsuki_iceberg_cleave_damage_delta</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>tsuki/iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>iceberg_cleave</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>on_inspiration</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>damage_delta</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>-20</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat(cards): add Tsuki stance deck data
</commit_message>
<xml_diff>
--- a/project-a/tables/excel/CharacterCards.xlsx
+++ b/project-a/tables/excel/CharacterCards.xlsx
@@ -415,12 +415,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>tsuki/long_sword_slash</t>
+          <t>tsuki/crescent_slash</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -605,12 +605,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>long_sword_slash</t>
+          <t>crescent_slash</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>장검 베기</t>
+          <t>초승 베기</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -628,18 +628,24 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>피해 {0}%.</t>
+          <t>피해 {0}%.
+[월영] 실드 {1}%.
+[참월] 피해 +{2}%.</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>2</v>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>월영,참월</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>tsuki/high_speed_slash</t>
+          <t>tsuki/flow_guard</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -649,41 +655,47 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>high_speed_slash</t>
+          <t>flow_guard</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>고속 베기</t>
+          <t>흐름 막기</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Attack</t>
+          <t>Idle</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>피해 {0}%.</t>
+          <t>실드 {0}%.
+[월영] 카드 {1}장 뽑기.
+[참월] 이번 턴 공격 피해 +{2}%.</t>
         </is>
       </c>
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>월영,참월</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>tsuki/let_flow</t>
+          <t>tsuki/stance_shift</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -693,16 +705,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>let_flow</t>
+          <t>stance_shift</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>흘려 보내기</t>
+          <t>자세 변경</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -716,18 +728,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>실드 {0}%.</t>
+          <t>[보존] 현재 자세를 반대 자세로 변경.
+[월영] 카드 {0}장 뽑기.
+[참월] 이번 턴 공격 피해 +{1}%.</t>
         </is>
       </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>보존,월영,참월</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>tsuki/suppress_ready</t>
+          <t>tsuki/afterimage_thrust</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -737,41 +755,47 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>suppress_ready</t>
+          <t>afterimage_thrust</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>제압 준비</t>
+          <t>달 가르기</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Idle</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>자신의 공격 카드 드로우 {0}. {2}턴간 자신의 공격 카드 피해량 {1}% 증가.</t>
+          <t>피해 {0}%를 2회.
+[월영] 자세 변경 카드 {1}장 생성.
+[참월] 피해 {2}%를 1회 추가.</t>
         </is>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>월영,참월</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>tsuki/steal_slash</t>
+          <t>tsuki/breath_reset</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -781,30 +805,32 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steal_slash</t>
+          <t>breath_reset</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>훔쳐베기</t>
+          <t>숨 고르기</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Attack</t>
+          <t>Idle</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>모든 적 피해 {0}%. 영감: 비용 {1} 감소.</t>
+          <t>카드 {0}장 뽑기.
+[월영] 실드 {1}%.
+[참월] 행동 포인트 {2} 획득.</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -812,14 +838,14 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>영감</t>
+          <t>월영,참월</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>tsuki/feint_strike</t>
+          <t>tsuki/rupture_cleave</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -829,16 +855,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>feint_strike</t>
+          <t>rupture_cleave</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>눈속임 일격</t>
+          <t>파열참</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -852,7 +878,9 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>[보존] 피해 {0}%. 핸드의 무작위 자신의 카드 {1}장의 영감 효과를 활성화.</t>
+          <t>모든 적 피해 {0}%.
+[월영] 실드 {1}%.
+[참월] {2}회 추가 타격.</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -860,14 +888,14 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>보존</t>
+          <t>월영,참월</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>tsuki/freezing_blade</t>
+          <t>tsuki/halfmoon_combo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -877,30 +905,32 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>freezing_blade</t>
+          <t>halfmoon_combo</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>빙점 칼날</t>
+          <t>반월 연격</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>enhance</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Idle</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>[유일] 자신의 영감 효과가 활성화된 카드 사용 시 모든 적에게 피해 {0}%.</t>
+          <t>피해 {0}%를 3회.
+[월영] 자세 변경 카드 {1}장 생성.
+[참월] 이번 턴 자세를 변경했다면 피해 +{2}%.</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -908,55 +938,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>유일</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>tsuki/iceberg_cleave</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>tsuki</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>iceberg_cleave</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>빙산 가르기</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>attack</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Attack</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>모든 적 피해 {0}%. 영감: 타격 {1}회 추가, 피해량 {2}% 감소.</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>영감</t>
+          <t>월영,참월</t>
         </is>
       </c>
     </row>
@@ -971,24 +953,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -1026,60 +1008,55 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>stance</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>effect_type</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>card_type</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>buff</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>duration_turns</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>child_effect_type</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>child_target</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
-        <is>
-          <t>child_percent</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
         <is>
           <t>text_arg_index</t>
         </is>
@@ -1113,60 +1090,55 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>string,null</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>string</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>string,null</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>string,null</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>string,null</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>int,null</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>int,null</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>int,null</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>string,null</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>string,null</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>string,null</t>
-        </is>
-      </c>
       <c r="Q3" t="inlineStr">
-        <is>
-          <t>int,null</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
         <is>
           <t>int,null</t>
         </is>
@@ -1253,21 +1225,16 @@
           <t>data</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>tsuki_long_sword_slash_damage</t>
+          <t>tsuki_crescent_slash_damage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>tsuki/long_sword_slash</t>
+          <t>tsuki/crescent_slash</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1277,7 +1244,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>long_sword_slash</t>
+          <t>crescent_slash</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1285,32 +1252,32 @@
           <t>on_play</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>enemy</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>100</v>
       </c>
-      <c r="R5" t="n">
+      <c r="Q5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>tsuki_high_speed_slash_damage</t>
+          <t>tsuki_crescent_slash_moon_shield</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>tsuki/high_speed_slash</t>
+          <t>tsuki/crescent_slash</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1320,40 +1287,45 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>high_speed_slash</t>
+          <t>crescent_slash</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>월영</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>enemy</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>220</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>tsuki_let_flow_shield</t>
+          <t>tsuki_crescent_slash_sun_damage_up</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>tsuki/let_flow</t>
+          <t>tsuki/crescent_slash</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1363,40 +1335,40 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>let_flow</t>
+          <t>crescent_slash</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>참월</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>100</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
+          <t>damage_delta</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>tsuki_suppress_ready_draw</t>
+          <t>tsuki_flow_guard_shield</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tsuki/suppress_ready</t>
+          <t>tsuki/flow_guard</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1406,7 +1378,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>suppress_ready</t>
+          <t>flow_guard</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1414,32 +1386,32 @@
           <t>on_play</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>draw</t>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>shield</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>self</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>tsuki_suppress_ready_attack_buff</t>
+          <t>tsuki_flow_guard_moon_draw</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tsuki/suppress_ready</t>
+          <t>tsuki/flow_guard</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1449,48 +1421,40 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>suppress_ready</t>
+          <t>flow_guard</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>buff</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>attack_damage_up</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>40</v>
+          <t>월영</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
       </c>
       <c r="M9" t="n">
         <v>1</v>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>own_attack</t>
-        </is>
-      </c>
-      <c r="R9" t="n">
+      <c r="Q9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>tsuki_suppress_ready_buff_turns_text</t>
+          <t>tsuki_flow_guard_sun_buff</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tsuki/suppress_ready</t>
+          <t>tsuki/flow_guard</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1500,35 +1464,45 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>suppress_ready</t>
+          <t>flow_guard</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>text_only</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>참월</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>buff</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>attack_damage_up</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q10" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>tsuki_steal_slash_damage</t>
+          <t>tsuki_stance_shift_change</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tsuki/steal_slash</t>
+          <t>tsuki/stance_shift</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1538,7 +1512,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>steal_slash</t>
+          <t>stance_shift</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1546,32 +1520,21 @@
           <t>on_play</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>damage</t>
-        </is>
-      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>all_enemies</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>220</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
+          <t>stance_change</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>tsuki_steal_slash_inspiration_cost</t>
+          <t>tsuki_stance_shift_moon_draw</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>tsuki/steal_slash</t>
+          <t>tsuki/stance_shift</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1581,35 +1544,40 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>steal_slash</t>
+          <t>stance_shift</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>on_inspiration</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>cost_delta</t>
-        </is>
-      </c>
-      <c r="L12" t="n">
-        <v>-1</v>
-      </c>
-      <c r="R12" t="n">
+          <t>월영</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
         <v>1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>tsuki_feint_strike_damage</t>
+          <t>tsuki_stance_shift_sun_buff</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tsuki/feint_strike</t>
+          <t>tsuki/stance_shift</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1619,40 +1587,45 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>feint_strike</t>
+          <t>stance_shift</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>참월</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>enemy</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>180</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
+          <t>buff</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>attack_damage_up</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>tsuki_feint_strike_activate_inspiration</t>
+          <t>tsuki_afterimage_thrust_damage_1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>tsuki/feint_strike</t>
+          <t>tsuki/afterimage_thrust</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1662,7 +1635,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>feint_strike</t>
+          <t>afterimage_thrust</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1670,32 +1643,32 @@
           <t>on_play</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>activate_inspiration</t>
-        </is>
-      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>random_own_in_hand</t>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>enemy</t>
         </is>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
-      </c>
-      <c r="R14" t="n">
-        <v>1</v>
+        <v>80</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>tsuki_freezing_blade_passive_damage</t>
+          <t>tsuki_afterimage_thrust_damage_2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tsuki/freezing_blade</t>
+          <t>tsuki/afterimage_thrust</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1705,40 +1678,37 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>freezing_blade</t>
+          <t>afterimage_thrust</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>on_play_inspired_card</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>all_enemies</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>120</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>tsuki_iceberg_cleave_damage</t>
+          <t>tsuki_afterimage_thrust_moon_add_stance</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>tsuki/iceberg_cleave</t>
+          <t>tsuki/afterimage_thrust</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1748,40 +1718,45 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>iceberg_cleave</t>
+          <t>afterimage_thrust</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>on_play</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>월영</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>all_enemies</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>180</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0</v>
+          <t>add_card_to_hand</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>stance_shift</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>tsuki_iceberg_cleave_extra_hit</t>
+          <t>tsuki_afterimage_thrust_sun_extra_damage</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>tsuki/iceberg_cleave</t>
+          <t>tsuki/afterimage_thrust</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1791,35 +1766,48 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>iceberg_cleave</t>
+          <t>afterimage_thrust</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>on_inspiration</t>
+          <t>on_stance</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>add_hit</t>
+          <t>참월</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>enemy</t>
         </is>
       </c>
       <c r="L17" t="n">
+        <v>80</v>
+      </c>
+      <c r="M17" t="n">
         <v>1</v>
       </c>
-      <c r="R17" t="n">
-        <v>1</v>
+      <c r="Q17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>tsuki_iceberg_cleave_damage_delta</t>
+          <t>tsuki_breath_reset_draw</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tsuki/iceberg_cleave</t>
+          <t>tsuki/breath_reset</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1829,23 +1817,467 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>iceberg_cleave</t>
+          <t>breath_reset</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>on_inspiration</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tsuki_breath_reset_moon_shield</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>tsuki/breath_reset</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>breath_reset</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>on_stance</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>월영</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tsuki_breath_reset_sun_energy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>tsuki/breath_reset</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>breath_reset</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>on_stance</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>참월</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tsuki_rupture_cleave_damage</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>tsuki/rupture_cleave</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>rupture_cleave</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>all_enemies</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>tsuki_rupture_cleave_moon_shield</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>tsuki/rupture_cleave</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>rupture_cleave</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>on_stance</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>월영</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tsuki_rupture_cleave_sun_add_hit</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>tsuki/rupture_cleave</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>rupture_cleave</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>on_stance</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>참월</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>add_hit</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tsuki_halfmoon_combo_damage_1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>tsuki/halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tsuki_halfmoon_combo_damage_2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>tsuki/halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>tsuki_halfmoon_combo_damage_3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>tsuki/halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>on_play</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>tsuki_halfmoon_combo_moon_add_stance</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>tsuki/halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>on_stance</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>월영</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>add_card_to_hand</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>stance_shift</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tsuki_halfmoon_combo_sun_damage_up</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tsuki/halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>tsuki</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>halfmoon_combo</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>on_stance</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>참월</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>damage_delta</t>
         </is>
       </c>
-      <c r="K18" t="n">
-        <v>-20</v>
-      </c>
-      <c r="R18" t="n">
+      <c r="L28" t="n">
+        <v>30</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>stance_changed_this_turn</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>